<commit_message>
Updated A-A filters w/ final version, updated BOM
</commit_message>
<xml_diff>
--- a/PCB/DAQBoardFront/BOM_DAQ.xlsx
+++ b/PCB/DAQBoardFront/BOM_DAQ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a56d338d63da0fa/Desktop/CFR-2027/PCB/DAQBoardFront/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="8_{672BEF6D-422F-477B-B486-B83020C6D7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D5788CA-3AD7-40EE-8EF9-A971D66E3DFC}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="8_{672BEF6D-422F-477B-B486-B83020C6D7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD1300AD-9901-4271-A29F-34D2B4B6F193}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{93B5DAD3-BF6B-4E2E-A13F-1D74895200EB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{93B5DAD3-BF6B-4E2E-A13F-1D74895200EB}"/>
   </bookViews>
   <sheets>
     <sheet name="DAQBoardFront" sheetId="2" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="95">
   <si>
     <t>Designator</t>
   </si>
@@ -127,21 +127,9 @@
     <t>53375-0410</t>
   </si>
   <si>
-    <t>L1, L2</t>
-  </si>
-  <si>
     <t>L_0805_2012Metric_Pad1.05x1.20mm_HandSolder</t>
   </si>
   <si>
-    <t>10u</t>
-  </si>
-  <si>
-    <t>L3</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
     <t>L4</t>
   </si>
   <si>
@@ -157,12 +145,6 @@
     <t>R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</t>
   </si>
   <si>
-    <t>1.69k</t>
-  </si>
-  <si>
-    <t>R3, R6</t>
-  </si>
-  <si>
     <t>R</t>
   </si>
   <si>
@@ -298,15 +280,9 @@
     <t>C5210749</t>
   </si>
   <si>
-    <t>C76742</t>
-  </si>
-  <si>
     <t>C2847484</t>
   </si>
   <si>
-    <t>C22846</t>
-  </si>
-  <si>
     <t>C23352</t>
   </si>
   <si>
@@ -332,6 +308,33 @@
   </si>
   <si>
     <t>C411212</t>
+  </si>
+  <si>
+    <t>6.57k</t>
+  </si>
+  <si>
+    <t>C861535</t>
+  </si>
+  <si>
+    <t>R6</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>22u</t>
+  </si>
+  <si>
+    <t>L1, L2, L3</t>
+  </si>
+  <si>
+    <t>C861266</t>
+  </si>
+  <si>
+    <t>26.4k</t>
+  </si>
+  <si>
+    <t>C88185</t>
   </si>
 </sst>
 </file>
@@ -714,7 +717,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -723,12 +726,12 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -737,12 +740,12 @@
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
@@ -751,7 +754,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -776,12 +779,12 @@
         <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
@@ -790,7 +793,7 @@
         <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -804,7 +807,7 @@
         <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -818,7 +821,7 @@
         <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -845,186 +848,189 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
       <c r="B11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11" t="s">
         <v>25</v>
       </c>
-      <c r="C11" t="s">
-        <v>26</v>
-      </c>
       <c r="D11" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="D12" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" t="s">
         <v>30</v>
       </c>
-      <c r="C13" t="s">
-        <v>31</v>
-      </c>
       <c r="D13" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>93</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
+        <v>89</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D14" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>88</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D16" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C17" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D17" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C18" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D18" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B19" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C19" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D19" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B20" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C20" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C21" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B22" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C22" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D22" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C23" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D23" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B24" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C24" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D24" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
@@ -1032,10 +1038,10 @@
         <v>21</v>
       </c>
       <c r="B25" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C25" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -1043,13 +1049,13 @@
         <v>21</v>
       </c>
       <c r="B26" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C26" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D26" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
@@ -1057,10 +1063,10 @@
         <v>21</v>
       </c>
       <c r="B27" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C27" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -1068,24 +1074,24 @@
         <v>21</v>
       </c>
       <c r="B28" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C28" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B29" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C29" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D29" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>